<commit_message>
feat(ventas): endpoint POST /ventas funcional
</commit_message>
<xml_diff>
--- a/data/datos.xlsx
+++ b/data/datos.xlsx
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <si>
     <t>Código</t>
   </si>
@@ -172,13 +172,29 @@
   </si>
   <si>
     <t>Procesado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4607900001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-02-25T16:20:19.639Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Laptop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mouse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Teclado</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts/>
+  <fonts x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -194,7 +210,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills>
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -207,7 +223,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders>
     <border>
       <left/>
       <right/>
@@ -220,7 +236,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -618,7 +634,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38113A1C-B25C-45F8-90F0-F3D668297EF0}">
-  <dimension ref="A1:J2"/>
+  <sheetPr/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" style="1" customWidth="1"/>
@@ -634,48 +650,132 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" t="s" s="3">
         <v>37</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" t="s" s="3">
         <v>35</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" t="s" s="3">
         <v>39</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" t="s" s="3">
         <v>34</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" t="s" s="3">
         <v>36</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" t="s" s="3">
         <v>40</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" t="s" s="3">
         <v>41</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" t="s" s="3">
         <v>42</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" t="s" s="3">
         <v>38</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" t="s" s="4">
         <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="4"/>
+      <c r="A2" t="s" s="3">
+        <v>44</v>
+      </c>
+      <c r="B2" t="s" s="3">
+        <v>45</v>
+      </c>
+      <c r="C2" s="3">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s" s="3">
+        <v>46</v>
+      </c>
+      <c r="E2" s="3">
+        <v>2</v>
+      </c>
+      <c r="F2" s="3">
+        <v>800</v>
+      </c>
+      <c r="G2" s="3">
+        <v>1600</v>
+      </c>
+      <c r="H2" s="3">
+        <v>1000</v>
+      </c>
+      <c r="I2" s="3">
+        <v>670</v>
+      </c>
+      <c r="J2" t="b" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="1">
+        <v>44</v>
+      </c>
+      <c r="B3" t="s" s="1">
+        <v>45</v>
+      </c>
+      <c r="C3" s="1">
+        <v>2</v>
+      </c>
+      <c r="D3" t="s" s="1">
+        <v>47</v>
+      </c>
+      <c r="E3" s="1">
+        <v>1</v>
+      </c>
+      <c r="F3" s="1">
+        <v>25</v>
+      </c>
+      <c r="G3" s="1">
+        <v>25</v>
+      </c>
+      <c r="H3" s="1">
+        <v>1000</v>
+      </c>
+      <c r="I3" s="1">
+        <v>670</v>
+      </c>
+      <c r="J3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="1">
+        <v>44</v>
+      </c>
+      <c r="B4" t="s" s="1">
+        <v>45</v>
+      </c>
+      <c r="C4" s="1">
+        <v>3</v>
+      </c>
+      <c r="D4" t="s" s="1">
+        <v>48</v>
+      </c>
+      <c r="E4" s="1">
+        <v>1</v>
+      </c>
+      <c r="F4" s="1">
+        <v>45</v>
+      </c>
+      <c r="G4" s="1">
+        <v>45</v>
+      </c>
+      <c r="H4" s="1">
+        <v>1000</v>
+      </c>
+      <c r="I4" s="1">
+        <v>670</v>
+      </c>
+      <c r="J4" t="b">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -687,7 +787,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D16"/>
+  <sheetPr/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.28515625" style="1" customWidth="1"/>
@@ -697,24 +797,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" t="s" s="2">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" t="s" s="2">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" t="s" s="2">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" t="s" s="2">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s" s="1">
         <v>4</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s" s="1">
         <v>19</v>
       </c>
       <c r="C2" s="1">
@@ -725,10 +825,10 @@
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" t="s" s="1">
         <v>5</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s" s="1">
         <v>20</v>
       </c>
       <c r="C3" s="1">
@@ -739,10 +839,10 @@
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s" s="1">
         <v>6</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s" s="1">
         <v>21</v>
       </c>
       <c r="C4" s="1">
@@ -753,10 +853,10 @@
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="A5" t="s" s="1">
         <v>7</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s" s="1">
         <v>22</v>
       </c>
       <c r="C5" s="1">
@@ -767,10 +867,10 @@
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="A6" t="s" s="1">
         <v>8</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s" s="1">
         <v>23</v>
       </c>
       <c r="C6" s="1">
@@ -781,10 +881,10 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="A7" t="s" s="1">
         <v>9</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s" s="1">
         <v>24</v>
       </c>
       <c r="C7" s="1">
@@ -795,10 +895,10 @@
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+      <c r="A8" t="s" s="1">
         <v>10</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s" s="1">
         <v>25</v>
       </c>
       <c r="C8" s="1">
@@ -809,10 +909,10 @@
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+      <c r="A9" t="s" s="1">
         <v>11</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" t="s" s="1">
         <v>26</v>
       </c>
       <c r="C9" s="1">
@@ -823,10 +923,10 @@
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+      <c r="A10" t="s" s="1">
         <v>12</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" t="s" s="1">
         <v>27</v>
       </c>
       <c r="C10" s="1">
@@ -837,10 +937,10 @@
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+      <c r="A11" t="s" s="1">
         <v>13</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" t="s" s="1">
         <v>28</v>
       </c>
       <c r="C11" s="1">
@@ -851,10 +951,10 @@
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+      <c r="A12" t="s" s="1">
         <v>14</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" t="s" s="1">
         <v>29</v>
       </c>
       <c r="C12" s="1">
@@ -865,10 +965,10 @@
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
+      <c r="A13" t="s" s="1">
         <v>15</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" t="s" s="1">
         <v>30</v>
       </c>
       <c r="C13" s="1">
@@ -879,10 +979,10 @@
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
+      <c r="A14" t="s" s="1">
         <v>16</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" t="s" s="1">
         <v>31</v>
       </c>
       <c r="C14" s="1">
@@ -893,10 +993,10 @@
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
+      <c r="A15" t="s" s="1">
         <v>17</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" t="s" s="1">
         <v>32</v>
       </c>
       <c r="C15" s="1">
@@ -907,10 +1007,10 @@
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
+      <c r="A16" t="s" s="1">
         <v>18</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" t="s" s="1">
         <v>33</v>
       </c>
       <c r="C16" s="1">

</xml_diff>

<commit_message>
se desarrolla la funcion de actualizar stock y se desarrollaron los botones de disminuir cantidades
</commit_message>
<xml_diff>
--- a/data/datos.xlsx
+++ b/data/datos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aris\Desktop\webapp-beta\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2931282-BCB9-4DAD-A66E-CB917CC4932E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC05925B-861C-4D84-ADFC-F2D5DE03DF23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}" activeTab="0"/>
   </bookViews>
@@ -174,10 +174,10 @@
     <t>Procesado</t>
   </si>
   <si>
-    <t xml:space="preserve">4607900001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-02-25T20:06:20.231Z</t>
+    <t xml:space="preserve">4608000001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-02-26T19:33:35.334Z</t>
   </si>
 </sst>
 </file>
@@ -695,7 +695,7 @@
         <v>990</v>
       </c>
       <c r="H2" s="3">
-        <v>2320</v>
+        <v>1670</v>
       </c>
       <c r="I2" s="3">
         <v>0</v>
@@ -712,22 +712,22 @@
         <v>45</v>
       </c>
       <c r="C3" t="s" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D3" t="s" s="1">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E3" s="1">
         <v>1</v>
       </c>
       <c r="F3" s="1">
-        <v>210</v>
+        <v>550</v>
       </c>
       <c r="G3" s="1">
-        <v>210</v>
+        <v>550</v>
       </c>
       <c r="H3" s="1">
-        <v>2320</v>
+        <v>1670</v>
       </c>
       <c r="I3" s="1">
         <v>0</v>
@@ -744,91 +744,27 @@
         <v>45</v>
       </c>
       <c r="C4" t="s" s="1">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D4" t="s" s="1">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="E4" s="1">
         <v>1</v>
       </c>
       <c r="F4" s="1">
-        <v>400</v>
+        <v>130</v>
       </c>
       <c r="G4" s="1">
-        <v>400</v>
+        <v>130</v>
       </c>
       <c r="H4" s="1">
-        <v>2320</v>
+        <v>1670</v>
       </c>
       <c r="I4" s="1">
         <v>0</v>
       </c>
       <c r="J4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s" s="1">
-        <v>44</v>
-      </c>
-      <c r="B5" t="s" s="1">
-        <v>45</v>
-      </c>
-      <c r="C5" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="D5" t="s" s="1">
-        <v>26</v>
-      </c>
-      <c r="E5" s="1">
-        <v>1</v>
-      </c>
-      <c r="F5" s="1">
-        <v>420</v>
-      </c>
-      <c r="G5" s="1">
-        <v>420</v>
-      </c>
-      <c r="H5" s="1">
-        <v>2320</v>
-      </c>
-      <c r="I5" s="1">
-        <v>0</v>
-      </c>
-      <c r="J5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s" s="1">
-        <v>44</v>
-      </c>
-      <c r="B6" t="s" s="1">
-        <v>45</v>
-      </c>
-      <c r="C6" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="D6" t="s" s="1">
-        <v>28</v>
-      </c>
-      <c r="E6" s="1">
-        <v>2</v>
-      </c>
-      <c r="F6" s="1">
-        <v>150</v>
-      </c>
-      <c r="G6" s="1">
-        <v>300</v>
-      </c>
-      <c r="H6" s="1">
-        <v>2320</v>
-      </c>
-      <c r="I6" s="1">
-        <v>0</v>
-      </c>
-      <c r="J6" t="b">
         <v>0</v>
       </c>
     </row>
@@ -873,7 +809,7 @@
         <v>19</v>
       </c>
       <c r="C2" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D2" s="1">
         <v>990</v>
@@ -887,7 +823,7 @@
         <v>20</v>
       </c>
       <c r="C3" s="1">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D3" s="1">
         <v>550</v>
@@ -901,7 +837,7 @@
         <v>21</v>
       </c>
       <c r="C4" s="1">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D4" s="1">
         <v>130</v>

</xml_diff>

<commit_message>
diseño naranja y confirmacion de vuelto
</commit_message>
<xml_diff>
--- a/data/datos.xlsx
+++ b/data/datos.xlsx
@@ -178,6 +178,18 @@
   </si>
   <si>
     <t xml:space="preserve">2026-02-26T19:33:35.334Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4608000002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-02-26T20:42:11.671Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4608000003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-02-27T02:55:09.894Z</t>
   </si>
 </sst>
 </file>
@@ -673,8 +685,8 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" t="s" s="3">
-        <v>44</v>
+      <c r="A2" s="3">
+        <v>4608000001</v>
       </c>
       <c r="B2" t="s" s="3">
         <v>45</v>
@@ -705,8 +717,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s" s="1">
-        <v>44</v>
+      <c r="A3" s="1">
+        <v>4608000001</v>
       </c>
       <c r="B3" t="s" s="1">
         <v>45</v>
@@ -737,8 +749,8 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="s" s="1">
-        <v>44</v>
+      <c r="A4" s="1">
+        <v>4608000001</v>
       </c>
       <c r="B4" t="s" s="1">
         <v>45</v>
@@ -765,6 +777,102 @@
         <v>0</v>
       </c>
       <c r="J4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1">
+        <v>4608000002</v>
+      </c>
+      <c r="B5" t="s" s="1">
+        <v>47</v>
+      </c>
+      <c r="C5" t="s" s="1">
+        <v>5</v>
+      </c>
+      <c r="D5" t="s" s="1">
+        <v>20</v>
+      </c>
+      <c r="E5" s="1">
+        <v>2</v>
+      </c>
+      <c r="F5" s="1">
+        <v>550</v>
+      </c>
+      <c r="G5" s="1">
+        <v>1100</v>
+      </c>
+      <c r="H5" s="1">
+        <v>1360</v>
+      </c>
+      <c r="I5" s="1">
+        <v>0</v>
+      </c>
+      <c r="J5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1">
+        <v>4608000002</v>
+      </c>
+      <c r="B6" t="s" s="1">
+        <v>47</v>
+      </c>
+      <c r="C6" t="s" s="1">
+        <v>6</v>
+      </c>
+      <c r="D6" t="s" s="1">
+        <v>21</v>
+      </c>
+      <c r="E6" s="1">
+        <v>2</v>
+      </c>
+      <c r="F6" s="1">
+        <v>130</v>
+      </c>
+      <c r="G6" s="1">
+        <v>260</v>
+      </c>
+      <c r="H6" s="1">
+        <v>1360</v>
+      </c>
+      <c r="I6" s="1">
+        <v>0</v>
+      </c>
+      <c r="J6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="1">
+        <v>48</v>
+      </c>
+      <c r="B7" t="s" s="1">
+        <v>49</v>
+      </c>
+      <c r="C7" t="s" s="1">
+        <v>4</v>
+      </c>
+      <c r="D7" t="s" s="1">
+        <v>19</v>
+      </c>
+      <c r="E7" s="1">
+        <v>1</v>
+      </c>
+      <c r="F7" s="1">
+        <v>990</v>
+      </c>
+      <c r="G7" s="1">
+        <v>990</v>
+      </c>
+      <c r="H7" s="1">
+        <v>990</v>
+      </c>
+      <c r="I7" s="1">
+        <v>0</v>
+      </c>
+      <c r="J7" t="b">
         <v>0</v>
       </c>
     </row>
@@ -809,7 +917,7 @@
         <v>19</v>
       </c>
       <c r="C2" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D2" s="1">
         <v>990</v>
@@ -823,7 +931,7 @@
         <v>20</v>
       </c>
       <c r="C3" s="1">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="D3" s="1">
         <v>550</v>
@@ -837,7 +945,7 @@
         <v>21</v>
       </c>
       <c r="C4" s="1">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D4" s="1">
         <v>130</v>

</xml_diff>

<commit_message>
Implementacion de modal estetico
</commit_message>
<xml_diff>
--- a/data/datos.xlsx
+++ b/data/datos.xlsx
@@ -190,6 +190,12 @@
   </si>
   <si>
     <t xml:space="preserve">2026-02-27T02:55:09.894Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4608000004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-02-27T03:11:49.420Z</t>
   </si>
 </sst>
 </file>
@@ -845,8 +851,8 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="s" s="1">
-        <v>48</v>
+      <c r="A7" s="1">
+        <v>4608000003</v>
       </c>
       <c r="B7" t="s" s="1">
         <v>49</v>
@@ -873,6 +879,70 @@
         <v>0</v>
       </c>
       <c r="J7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="1">
+        <v>50</v>
+      </c>
+      <c r="B8" t="s" s="1">
+        <v>51</v>
+      </c>
+      <c r="C8" t="s" s="1">
+        <v>5</v>
+      </c>
+      <c r="D8" t="s" s="1">
+        <v>20</v>
+      </c>
+      <c r="E8" s="1">
+        <v>1</v>
+      </c>
+      <c r="F8" s="1">
+        <v>550</v>
+      </c>
+      <c r="G8" s="1">
+        <v>550</v>
+      </c>
+      <c r="H8" s="1">
+        <v>680</v>
+      </c>
+      <c r="I8" s="1">
+        <v>0</v>
+      </c>
+      <c r="J8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="1">
+        <v>50</v>
+      </c>
+      <c r="B9" t="s" s="1">
+        <v>51</v>
+      </c>
+      <c r="C9" t="s" s="1">
+        <v>6</v>
+      </c>
+      <c r="D9" t="s" s="1">
+        <v>21</v>
+      </c>
+      <c r="E9" s="1">
+        <v>1</v>
+      </c>
+      <c r="F9" s="1">
+        <v>130</v>
+      </c>
+      <c r="G9" s="1">
+        <v>130</v>
+      </c>
+      <c r="H9" s="1">
+        <v>680</v>
+      </c>
+      <c r="I9" s="1">
+        <v>0</v>
+      </c>
+      <c r="J9" t="b">
         <v>0</v>
       </c>
     </row>
@@ -931,7 +1001,7 @@
         <v>20</v>
       </c>
       <c r="C3" s="1">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="D3" s="1">
         <v>550</v>
@@ -945,7 +1015,7 @@
         <v>21</v>
       </c>
       <c r="C4" s="1">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D4" s="1">
         <v>130</v>

</xml_diff>

<commit_message>
Deshabilitado el boton de agregar cuando no hay stock
</commit_message>
<xml_diff>
--- a/data/datos.xlsx
+++ b/data/datos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aris\Desktop\webapp-beta\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC05925B-861C-4D84-ADFC-F2D5DE03DF23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FE6A4BD-197E-4DC1-A721-F9C7A232D2E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}" activeTab="0"/>
   </bookViews>
@@ -177,25 +177,13 @@
     <t xml:space="preserve">4608000001</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-02-26T19:33:35.334Z</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4608000002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-02-26T20:42:11.671Z</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4608000003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-02-27T02:55:09.894Z</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4608000004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-02-27T03:11:49.420Z</t>
+    <t xml:space="preserve">2026-02-27T03:42:50.752Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4608100001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-02-27T16:03:59.256Z</t>
   </si>
 </sst>
 </file>
@@ -704,16 +692,16 @@
         <v>19</v>
       </c>
       <c r="E2" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F2" s="3">
         <v>990</v>
       </c>
       <c r="G2" s="3">
-        <v>990</v>
+        <v>2970</v>
       </c>
       <c r="H2" s="3">
-        <v>1670</v>
+        <v>2970</v>
       </c>
       <c r="I2" s="3">
         <v>0</v>
@@ -723,11 +711,11 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1">
-        <v>4608000001</v>
+      <c r="A3" t="s" s="1">
+        <v>46</v>
       </c>
       <c r="B3" t="s" s="1">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C3" t="s" s="1">
         <v>5</v>
@@ -736,16 +724,16 @@
         <v>20</v>
       </c>
       <c r="E3" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F3" s="1">
         <v>550</v>
       </c>
       <c r="G3" s="1">
-        <v>550</v>
+        <v>1100</v>
       </c>
       <c r="H3" s="1">
-        <v>1670</v>
+        <v>1310</v>
       </c>
       <c r="I3" s="1">
         <v>0</v>
@@ -755,194 +743,34 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1">
-        <v>4608000001</v>
+      <c r="A4" t="s" s="1">
+        <v>46</v>
       </c>
       <c r="B4" t="s" s="1">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C4" t="s" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D4" t="s" s="1">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E4" s="1">
         <v>1</v>
       </c>
       <c r="F4" s="1">
-        <v>130</v>
+        <v>210</v>
       </c>
       <c r="G4" s="1">
-        <v>130</v>
+        <v>210</v>
       </c>
       <c r="H4" s="1">
-        <v>1670</v>
+        <v>1310</v>
       </c>
       <c r="I4" s="1">
         <v>0</v>
       </c>
       <c r="J4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1">
-        <v>4608000002</v>
-      </c>
-      <c r="B5" t="s" s="1">
-        <v>47</v>
-      </c>
-      <c r="C5" t="s" s="1">
-        <v>5</v>
-      </c>
-      <c r="D5" t="s" s="1">
-        <v>20</v>
-      </c>
-      <c r="E5" s="1">
-        <v>2</v>
-      </c>
-      <c r="F5" s="1">
-        <v>550</v>
-      </c>
-      <c r="G5" s="1">
-        <v>1100</v>
-      </c>
-      <c r="H5" s="1">
-        <v>1360</v>
-      </c>
-      <c r="I5" s="1">
-        <v>0</v>
-      </c>
-      <c r="J5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1">
-        <v>4608000002</v>
-      </c>
-      <c r="B6" t="s" s="1">
-        <v>47</v>
-      </c>
-      <c r="C6" t="s" s="1">
-        <v>6</v>
-      </c>
-      <c r="D6" t="s" s="1">
-        <v>21</v>
-      </c>
-      <c r="E6" s="1">
-        <v>2</v>
-      </c>
-      <c r="F6" s="1">
-        <v>130</v>
-      </c>
-      <c r="G6" s="1">
-        <v>260</v>
-      </c>
-      <c r="H6" s="1">
-        <v>1360</v>
-      </c>
-      <c r="I6" s="1">
-        <v>0</v>
-      </c>
-      <c r="J6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1">
-        <v>4608000003</v>
-      </c>
-      <c r="B7" t="s" s="1">
-        <v>49</v>
-      </c>
-      <c r="C7" t="s" s="1">
-        <v>4</v>
-      </c>
-      <c r="D7" t="s" s="1">
-        <v>19</v>
-      </c>
-      <c r="E7" s="1">
-        <v>1</v>
-      </c>
-      <c r="F7" s="1">
-        <v>990</v>
-      </c>
-      <c r="G7" s="1">
-        <v>990</v>
-      </c>
-      <c r="H7" s="1">
-        <v>990</v>
-      </c>
-      <c r="I7" s="1">
-        <v>0</v>
-      </c>
-      <c r="J7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s" s="1">
-        <v>50</v>
-      </c>
-      <c r="B8" t="s" s="1">
-        <v>51</v>
-      </c>
-      <c r="C8" t="s" s="1">
-        <v>5</v>
-      </c>
-      <c r="D8" t="s" s="1">
-        <v>20</v>
-      </c>
-      <c r="E8" s="1">
-        <v>1</v>
-      </c>
-      <c r="F8" s="1">
-        <v>550</v>
-      </c>
-      <c r="G8" s="1">
-        <v>550</v>
-      </c>
-      <c r="H8" s="1">
-        <v>680</v>
-      </c>
-      <c r="I8" s="1">
-        <v>0</v>
-      </c>
-      <c r="J8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s" s="1">
-        <v>50</v>
-      </c>
-      <c r="B9" t="s" s="1">
-        <v>51</v>
-      </c>
-      <c r="C9" t="s" s="1">
-        <v>6</v>
-      </c>
-      <c r="D9" t="s" s="1">
-        <v>21</v>
-      </c>
-      <c r="E9" s="1">
-        <v>1</v>
-      </c>
-      <c r="F9" s="1">
-        <v>130</v>
-      </c>
-      <c r="G9" s="1">
-        <v>130</v>
-      </c>
-      <c r="H9" s="1">
-        <v>680</v>
-      </c>
-      <c r="I9" s="1">
-        <v>0</v>
-      </c>
-      <c r="J9" t="b">
         <v>0</v>
       </c>
     </row>
@@ -987,7 +815,7 @@
         <v>19</v>
       </c>
       <c r="C2" s="1">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D2" s="1">
         <v>990</v>
@@ -1001,7 +829,7 @@
         <v>20</v>
       </c>
       <c r="C3" s="1">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="D3" s="1">
         <v>550</v>
@@ -1029,7 +857,7 @@
         <v>22</v>
       </c>
       <c r="C5" s="1">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D5" s="1">
         <v>210</v>

</xml_diff>

<commit_message>
Generar factura corregido con eliminacion del ajuste de 1900
</commit_message>
<xml_diff>
--- a/data/datos.xlsx
+++ b/data/datos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aris\Desktop\webapp-beta\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FE6A4BD-197E-4DC1-A721-F9C7A232D2E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAB8D553-748F-4FFD-9986-572431052A56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}" activeTab="0"/>
   </bookViews>
@@ -174,16 +174,10 @@
     <t>Procesado</t>
   </si>
   <si>
-    <t xml:space="preserve">4608000001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-02-27T03:42:50.752Z</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4608100001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-02-27T16:03:59.256Z</t>
+    <t xml:space="preserve">4608200001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-03-01T20:51:42.377Z</t>
   </si>
 </sst>
 </file>
@@ -635,7 +629,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="26.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="29.85546875" style="1" customWidth="1"/>
     <col min="3" max="3" width="20.42578125" style="1" customWidth="1"/>
     <col min="4" max="4" width="23" style="1" customWidth="1"/>
     <col min="5" max="5" width="18.85546875" style="1" customWidth="1"/>
@@ -679,29 +673,29 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="3">
-        <v>4608000001</v>
+      <c r="A2" t="s" s="3">
+        <v>44</v>
       </c>
       <c r="B2" t="s" s="3">
         <v>45</v>
       </c>
       <c r="C2" t="s" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D2" t="s" s="3">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E2" s="3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F2" s="3">
-        <v>990</v>
+        <v>550</v>
       </c>
       <c r="G2" s="3">
-        <v>2970</v>
+        <v>550</v>
       </c>
       <c r="H2" s="3">
-        <v>2970</v>
+        <v>680</v>
       </c>
       <c r="I2" s="3">
         <v>0</v>
@@ -712,65 +706,33 @@
     </row>
     <row r="3">
       <c r="A3" t="s" s="1">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B3" t="s" s="1">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C3" t="s" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D3" t="s" s="1">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E3" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F3" s="1">
-        <v>550</v>
+        <v>130</v>
       </c>
       <c r="G3" s="1">
-        <v>1100</v>
+        <v>130</v>
       </c>
       <c r="H3" s="1">
-        <v>1310</v>
+        <v>680</v>
       </c>
       <c r="I3" s="1">
         <v>0</v>
       </c>
       <c r="J3" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s" s="1">
-        <v>46</v>
-      </c>
-      <c r="B4" t="s" s="1">
-        <v>47</v>
-      </c>
-      <c r="C4" t="s" s="1">
-        <v>7</v>
-      </c>
-      <c r="D4" t="s" s="1">
-        <v>22</v>
-      </c>
-      <c r="E4" s="1">
-        <v>1</v>
-      </c>
-      <c r="F4" s="1">
-        <v>210</v>
-      </c>
-      <c r="G4" s="1">
-        <v>210</v>
-      </c>
-      <c r="H4" s="1">
-        <v>1310</v>
-      </c>
-      <c r="I4" s="1">
-        <v>0</v>
-      </c>
-      <c r="J4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -829,7 +791,7 @@
         <v>20</v>
       </c>
       <c r="C3" s="1">
-        <v>291</v>
+        <v>284</v>
       </c>
       <c r="D3" s="1">
         <v>550</v>
@@ -843,7 +805,7 @@
         <v>21</v>
       </c>
       <c r="C4" s="1">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="D4" s="1">
         <v>130</v>
@@ -857,7 +819,7 @@
         <v>22</v>
       </c>
       <c r="C5" s="1">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D5" s="1">
         <v>210</v>
@@ -871,7 +833,7 @@
         <v>23</v>
       </c>
       <c r="C6" s="1">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D6" s="1">
         <v>180</v>
@@ -899,7 +861,7 @@
         <v>25</v>
       </c>
       <c r="C8" s="1">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D8" s="1">
         <v>850</v>
@@ -913,7 +875,7 @@
         <v>26</v>
       </c>
       <c r="C9" s="1">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D9" s="1">
         <v>420</v>
@@ -997,7 +959,7 @@
         <v>32</v>
       </c>
       <c r="C15" s="1">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D15" s="1">
         <v>60</v>
@@ -1011,7 +973,7 @@
         <v>33</v>
       </c>
       <c r="C16" s="1">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D16" s="1">
         <v>40</v>

</xml_diff>

<commit_message>
Configuracion de variables de entorno y preparacion para subir a github
</commit_message>
<xml_diff>
--- a/data/datos.xlsx
+++ b/data/datos.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
-  <workbookPr/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aris\Desktop\webapp-beta\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aris\Desktop\pos-movil\webapp-beta\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAB8D553-748F-4FFD-9986-572431052A56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCB98F75-8E03-46BF-9DEF-254B8A4F1F29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}" activeTab="0"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pendientes" sheetId="4" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="30">
   <si>
     <t>Código</t>
   </si>
@@ -54,138 +54,89 @@
     <t>Precio</t>
   </si>
   <si>
-    <t>Pr_00005</t>
+    <t>Nombre del producto</t>
+  </si>
+  <si>
+    <t>Fecha de venta</t>
+  </si>
+  <si>
+    <t>Cantidad Vendida</t>
+  </si>
+  <si>
+    <t>Factura ID</t>
+  </si>
+  <si>
+    <t>Transferencia</t>
+  </si>
+  <si>
+    <t>Código de producto</t>
+  </si>
+  <si>
+    <t>Precio unitario</t>
+  </si>
+  <si>
+    <t>Subtotal</t>
+  </si>
+  <si>
+    <t>Efectivo</t>
+  </si>
+  <si>
+    <t>Procesado</t>
+  </si>
+  <si>
+    <t>Pr_00014</t>
+  </si>
+  <si>
+    <t>Aceite</t>
   </si>
   <si>
     <t>Pr_00013</t>
   </si>
   <si>
-    <t>Pr_00010</t>
-  </si>
-  <si>
-    <t>Pr_00008</t>
-  </si>
-  <si>
-    <t>Pr_00006</t>
-  </si>
-  <si>
-    <t>Pr_00009</t>
-  </si>
-  <si>
-    <t>Pr_00002</t>
-  </si>
-  <si>
-    <t>Pr_00007</t>
-  </si>
-  <si>
-    <t>Pr_00012</t>
-  </si>
-  <si>
-    <t>Pr_00011</t>
-  </si>
-  <si>
-    <t>Pr_00003</t>
-  </si>
-  <si>
-    <t>Pr_00001</t>
-  </si>
-  <si>
-    <t>Pr_00004</t>
-  </si>
-  <si>
-    <t>Pr_00014</t>
+    <t>Azúcar x paquetes</t>
   </si>
   <si>
     <t>Pr_00015</t>
   </si>
   <si>
-    <t>Aceite</t>
-  </si>
-  <si>
-    <t>Azúcar x paquetes</t>
-  </si>
-  <si>
     <t>Donas de Fábrica</t>
   </si>
   <si>
-    <t>Galletas Dulces Rellenas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Galletas María </t>
+    <t>Pr_00016</t>
+  </si>
+  <si>
+    <t>Galletas dulces rellenas</t>
+  </si>
+  <si>
+    <t>Pr_00017</t>
+  </si>
+  <si>
+    <t>Galletas María</t>
+  </si>
+  <si>
+    <t>Pr_00018</t>
   </si>
   <si>
     <t>Ketchup</t>
   </si>
   <si>
-    <t>Marinado Agridulce</t>
-  </si>
-  <si>
-    <t>Mayonesa</t>
-  </si>
-  <si>
-    <t>Mentaplus</t>
-  </si>
-  <si>
-    <t>Paletas de Helado</t>
-  </si>
-  <si>
-    <t>Refresoc 2L</t>
+    <t>Pr_00019</t>
   </si>
   <si>
     <t>Sazón Goya</t>
   </si>
   <si>
-    <t>Sorbetos 80g</t>
-  </si>
-  <si>
-    <t>Rosquitas</t>
-  </si>
-  <si>
-    <t>Polvorón</t>
-  </si>
-  <si>
-    <t>Nombre del producto</t>
-  </si>
-  <si>
-    <t>Fecha de venta</t>
-  </si>
-  <si>
-    <t>Cantidad Vendida</t>
-  </si>
-  <si>
-    <t>Factura ID</t>
-  </si>
-  <si>
-    <t>Transferencia</t>
-  </si>
-  <si>
-    <t>Código de producto</t>
-  </si>
-  <si>
-    <t>Precio unitario</t>
-  </si>
-  <si>
-    <t>Subtotal</t>
-  </si>
-  <si>
-    <t>Efectivo</t>
-  </si>
-  <si>
-    <t>Procesado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4608200001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-03-01T20:51:42.377Z</t>
+    <t>4611700001</t>
+  </si>
+  <si>
+    <t>2026-04-05T21:19:47.312Z</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts/>
-  <fonts x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -201,7 +152,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills>
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -214,7 +165,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders>
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -227,7 +178,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs>
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -625,7 +576,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38113A1C-B25C-45F8-90F0-F3D668297EF0}">
-  <sheetPr/>
+  <sheetPr codeName="Hoja1"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" style="1" customWidth="1"/>
@@ -641,99 +593,67 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" t="s" s="3">
-        <v>37</v>
-      </c>
-      <c r="B1" t="s" s="3">
-        <v>35</v>
-      </c>
-      <c r="C1" t="s" s="3">
-        <v>39</v>
-      </c>
-      <c r="D1" t="s" s="3">
-        <v>34</v>
-      </c>
-      <c r="E1" t="s" s="3">
-        <v>36</v>
-      </c>
-      <c r="F1" t="s" s="3">
-        <v>40</v>
-      </c>
-      <c r="G1" t="s" s="3">
-        <v>41</v>
-      </c>
-      <c r="H1" t="s" s="3">
-        <v>42</v>
-      </c>
-      <c r="I1" t="s" s="3">
-        <v>38</v>
-      </c>
-      <c r="J1" t="s" s="4">
-        <v>43</v>
+      <c r="A1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" t="s" s="3">
-        <v>44</v>
-      </c>
-      <c r="B2" t="s" s="3">
-        <v>45</v>
-      </c>
-      <c r="C2" t="s" s="3">
-        <v>5</v>
-      </c>
-      <c r="D2" t="s" s="3">
-        <v>20</v>
+      <c r="A2" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="E2" s="3">
         <v>1</v>
       </c>
       <c r="F2" s="3">
-        <v>550</v>
+        <v>990</v>
       </c>
       <c r="G2" s="3">
-        <v>550</v>
+        <v>990</v>
       </c>
       <c r="H2" s="3">
-        <v>680</v>
+        <v>990</v>
       </c>
       <c r="I2" s="3">
         <v>0</v>
       </c>
-      <c r="J2" t="b" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s" s="1">
-        <v>44</v>
-      </c>
-      <c r="B3" t="s" s="1">
-        <v>45</v>
-      </c>
-      <c r="C3" t="s" s="1">
-        <v>6</v>
-      </c>
-      <c r="D3" t="s" s="1">
-        <v>21</v>
-      </c>
-      <c r="E3" s="1">
+      <c r="J2" s="4" t="b">
         <v>1</v>
-      </c>
-      <c r="F3" s="1">
-        <v>130</v>
-      </c>
-      <c r="G3" s="1">
-        <v>130</v>
-      </c>
-      <c r="H3" s="1">
-        <v>680</v>
-      </c>
-      <c r="I3" s="1">
-        <v>0</v>
-      </c>
-      <c r="J3" t="b">
-        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -746,7 +666,8 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr/>
+  <sheetPr codeName="Hoja2"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.28515625" style="1" customWidth="1"/>
@@ -756,53 +677,53 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s" s="2">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s" s="2">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s" s="2">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s" s="2">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s" s="1">
-        <v>4</v>
-      </c>
-      <c r="B2" t="s" s="1">
-        <v>19</v>
+      <c r="A2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>15</v>
       </c>
       <c r="C2" s="1">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="D2" s="1">
         <v>990</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s" s="1">
-        <v>5</v>
-      </c>
-      <c r="B3" t="s" s="1">
-        <v>20</v>
+      <c r="A3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>17</v>
       </c>
       <c r="C3" s="1">
-        <v>284</v>
+        <v>272</v>
       </c>
       <c r="D3" s="1">
         <v>550</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s" s="1">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s" s="1">
-        <v>21</v>
+      <c r="A4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>19</v>
       </c>
       <c r="C4" s="1">
         <v>75</v>
@@ -812,11 +733,11 @@
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s" s="1">
-        <v>7</v>
-      </c>
-      <c r="B5" t="s" s="1">
-        <v>22</v>
+      <c r="A5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>21</v>
       </c>
       <c r="C5" s="1">
         <v>45</v>
@@ -826,10 +747,10 @@
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s" s="1">
-        <v>8</v>
-      </c>
-      <c r="B6" t="s" s="1">
+      <c r="A6" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>23</v>
       </c>
       <c r="C6" s="1">
@@ -840,11 +761,11 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" t="s" s="1">
-        <v>9</v>
-      </c>
-      <c r="B7" t="s" s="1">
+      <c r="A7" s="1" t="s">
         <v>24</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="C7" s="1">
         <v>13</v>
@@ -854,129 +775,17 @@
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" t="s" s="1">
-        <v>10</v>
-      </c>
-      <c r="B8" t="s" s="1">
-        <v>25</v>
+      <c r="A8" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="C8" s="1">
-        <v>11</v>
+        <v>457</v>
       </c>
       <c r="D8" s="1">
-        <v>850</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="B9" t="s" s="1">
-        <v>26</v>
-      </c>
-      <c r="C9" s="1">
-        <v>18</v>
-      </c>
-      <c r="D9" s="1">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" t="s" s="1">
-        <v>12</v>
-      </c>
-      <c r="B10" t="s" s="1">
-        <v>27</v>
-      </c>
-      <c r="C10" s="1">
-        <v>198</v>
-      </c>
-      <c r="D10" s="1">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="B11" t="s" s="1">
-        <v>28</v>
-      </c>
-      <c r="C11" s="1">
-        <v>368</v>
-      </c>
-      <c r="D11" s="1">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" t="s" s="1">
-        <v>14</v>
-      </c>
-      <c r="B12" t="s" s="1">
-        <v>29</v>
-      </c>
-      <c r="C12" s="1">
-        <v>485</v>
-      </c>
-      <c r="D12" s="1">
         <v>30</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="B13" t="s" s="1">
-        <v>30</v>
-      </c>
-      <c r="C13" s="1">
-        <v>457</v>
-      </c>
-      <c r="D13" s="1">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" t="s" s="1">
-        <v>16</v>
-      </c>
-      <c r="B14" t="s" s="1">
-        <v>31</v>
-      </c>
-      <c r="C14" s="1">
-        <v>65</v>
-      </c>
-      <c r="D14" s="1">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" t="s" s="1">
-        <v>17</v>
-      </c>
-      <c r="B15" t="s" s="1">
-        <v>32</v>
-      </c>
-      <c r="C15" s="1">
-        <v>14</v>
-      </c>
-      <c r="D15" s="1">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" t="s" s="1">
-        <v>18</v>
-      </c>
-      <c r="B16" t="s" s="1">
-        <v>33</v>
-      </c>
-      <c r="C16" s="1">
-        <v>9</v>
-      </c>
-      <c r="D16" s="1">
-        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Añadí las carpetas flags y data al repositorio
</commit_message>
<xml_diff>
--- a/data/datos.xlsx
+++ b/data/datos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aris\Desktop\pos-movil\webapp-beta\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCB98F75-8E03-46BF-9DEF-254B8A4F1F29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C000460B-8DA3-465B-9B76-F384B20BE509}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>Código</t>
   </si>
@@ -88,42 +88,6 @@
   </si>
   <si>
     <t>Aceite</t>
-  </si>
-  <si>
-    <t>Pr_00013</t>
-  </si>
-  <si>
-    <t>Azúcar x paquetes</t>
-  </si>
-  <si>
-    <t>Pr_00015</t>
-  </si>
-  <si>
-    <t>Donas de Fábrica</t>
-  </si>
-  <si>
-    <t>Pr_00016</t>
-  </si>
-  <si>
-    <t>Galletas dulces rellenas</t>
-  </si>
-  <si>
-    <t>Pr_00017</t>
-  </si>
-  <si>
-    <t>Galletas María</t>
-  </si>
-  <si>
-    <t>Pr_00018</t>
-  </si>
-  <si>
-    <t>Ketchup</t>
-  </si>
-  <si>
-    <t>Pr_00019</t>
-  </si>
-  <si>
-    <t>Sazón Goya</t>
   </si>
   <si>
     <t>4611700001</t>
@@ -626,10 +590,10 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>14</v>
@@ -667,7 +631,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Hoja2"/>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.28515625" style="1" customWidth="1"/>
@@ -690,104 +654,6 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" s="1">
-        <v>9</v>
-      </c>
-      <c r="D2" s="1">
-        <v>990</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" s="1">
-        <v>272</v>
-      </c>
-      <c r="D3" s="1">
-        <v>550</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" s="1">
-        <v>75</v>
-      </c>
-      <c r="D4" s="1">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C5" s="1">
-        <v>45</v>
-      </c>
-      <c r="D5" s="1">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" s="1">
-        <v>44</v>
-      </c>
-      <c r="D6" s="1">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C7" s="1">
-        <v>13</v>
-      </c>
-      <c r="D7" s="1">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C8" s="1">
-        <v>457</v>
-      </c>
-      <c r="D8" s="1">
-        <v>30</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
se eliminaron datos residuales en la tabla
</commit_message>
<xml_diff>
--- a/data/datos.xlsx
+++ b/data/datos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aris\Desktop\pos-movil\webapp-beta\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C000460B-8DA3-465B-9B76-F384B20BE509}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2EEB289-56B6-4C7E-9F92-ECC0261D5331}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pendientes" sheetId="4" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Código</t>
   </si>
@@ -82,18 +82,6 @@
   </si>
   <si>
     <t>Procesado</t>
-  </si>
-  <si>
-    <t>Pr_00014</t>
-  </si>
-  <si>
-    <t>Aceite</t>
-  </si>
-  <si>
-    <t>4611700001</t>
-  </si>
-  <si>
-    <t>2026-04-05T21:19:47.312Z</t>
   </si>
 </sst>
 </file>
@@ -589,36 +577,16 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E2" s="3">
-        <v>1</v>
-      </c>
-      <c r="F2" s="3">
-        <v>990</v>
-      </c>
-      <c r="G2" s="3">
-        <v>990</v>
-      </c>
-      <c r="H2" s="3">
-        <v>990</v>
-      </c>
-      <c r="I2" s="3">
-        <v>0</v>
-      </c>
-      <c r="J2" s="4" t="b">
-        <v>1</v>
-      </c>
+      <c r="A2" s="3"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
corrección en desfase de fecha
</commit_message>
<xml_diff>
--- a/data/datos.xlsx
+++ b/data/datos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aris\Desktop\pos-movil\webapp-beta\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2EEB289-56B6-4C7E-9F92-ECC0261D5331}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12891C35-4278-46B1-B841-BF53021D3B5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="33">
   <si>
     <t>Código</t>
   </si>
@@ -82,6 +82,63 @@
   </si>
   <si>
     <t>Procesado</t>
+  </si>
+  <si>
+    <t>Pr_00014</t>
+  </si>
+  <si>
+    <t>Aceite</t>
+  </si>
+  <si>
+    <t>Pr_00013</t>
+  </si>
+  <si>
+    <t>Azúcar x paquetes</t>
+  </si>
+  <si>
+    <t>Pr_00015</t>
+  </si>
+  <si>
+    <t>Donas de Fábrica</t>
+  </si>
+  <si>
+    <t>Pr_00016</t>
+  </si>
+  <si>
+    <t>Galletas dulces rellenas</t>
+  </si>
+  <si>
+    <t>Pr_00017</t>
+  </si>
+  <si>
+    <t>Galletas María</t>
+  </si>
+  <si>
+    <t>Pr_00018</t>
+  </si>
+  <si>
+    <t>Ketchup</t>
+  </si>
+  <si>
+    <t>Pr_00019</t>
+  </si>
+  <si>
+    <t>Sazón Goya</t>
+  </si>
+  <si>
+    <t>2026-04-06T02:43:33.391Z</t>
+  </si>
+  <si>
+    <t>2026-04-06T13:10:00.224Z</t>
+  </si>
+  <si>
+    <t>2026-04-06T14:11:43.886-04:00</t>
+  </si>
+  <si>
+    <t>4611800004</t>
+  </si>
+  <si>
+    <t>2026-04-06T10:33:53.773</t>
   </si>
 </sst>
 </file>
@@ -529,7 +586,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38113A1C-B25C-45F8-90F0-F3D668297EF0}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" style="1" customWidth="1"/>
@@ -577,16 +634,228 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="4"/>
+      <c r="A2" s="3">
+        <v>4611800001</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" s="3">
+        <v>1</v>
+      </c>
+      <c r="F2" s="3">
+        <v>130</v>
+      </c>
+      <c r="G2" s="3">
+        <v>130</v>
+      </c>
+      <c r="H2" s="3">
+        <v>0</v>
+      </c>
+      <c r="I2" s="3">
+        <v>130</v>
+      </c>
+      <c r="J2" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
+        <v>4611800002</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E3" s="1">
+        <v>1</v>
+      </c>
+      <c r="F3" s="1">
+        <v>400</v>
+      </c>
+      <c r="G3" s="1">
+        <v>400</v>
+      </c>
+      <c r="H3" s="1">
+        <v>400</v>
+      </c>
+      <c r="I3" s="1">
+        <v>0</v>
+      </c>
+      <c r="J3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
+        <v>4611800003</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" s="1">
+        <v>1</v>
+      </c>
+      <c r="F4" s="1">
+        <v>30</v>
+      </c>
+      <c r="G4" s="1">
+        <v>30</v>
+      </c>
+      <c r="H4" s="1">
+        <v>580</v>
+      </c>
+      <c r="I4" s="1">
+        <v>0</v>
+      </c>
+      <c r="J4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
+        <v>4611800003</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" s="1">
+        <v>1</v>
+      </c>
+      <c r="F5" s="1">
+        <v>550</v>
+      </c>
+      <c r="G5" s="1">
+        <v>550</v>
+      </c>
+      <c r="H5" s="1">
+        <v>580</v>
+      </c>
+      <c r="I5" s="1">
+        <v>0</v>
+      </c>
+      <c r="J5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="1">
+        <v>1</v>
+      </c>
+      <c r="F6" s="1">
+        <v>130</v>
+      </c>
+      <c r="G6" s="1">
+        <v>130</v>
+      </c>
+      <c r="H6" s="1">
+        <v>710</v>
+      </c>
+      <c r="I6" s="1">
+        <v>0</v>
+      </c>
+      <c r="J6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E7" s="1">
+        <v>1</v>
+      </c>
+      <c r="F7" s="1">
+        <v>180</v>
+      </c>
+      <c r="G7" s="1">
+        <v>180</v>
+      </c>
+      <c r="H7" s="1">
+        <v>710</v>
+      </c>
+      <c r="I7" s="1">
+        <v>0</v>
+      </c>
+      <c r="J7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E8" s="1">
+        <v>1</v>
+      </c>
+      <c r="F8" s="1">
+        <v>400</v>
+      </c>
+      <c r="G8" s="1">
+        <v>400</v>
+      </c>
+      <c r="H8" s="1">
+        <v>710</v>
+      </c>
+      <c r="I8" s="1">
+        <v>0</v>
+      </c>
+      <c r="J8" t="b">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -599,7 +868,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Hoja2"/>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.28515625" style="1" customWidth="1"/>
@@ -622,6 +891,104 @@
         <v>3</v>
       </c>
     </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="1">
+        <v>10</v>
+      </c>
+      <c r="D2" s="1">
+        <v>990</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="1">
+        <v>272</v>
+      </c>
+      <c r="D3" s="1">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="1">
+        <v>74</v>
+      </c>
+      <c r="D4" s="1">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="1">
+        <v>45</v>
+      </c>
+      <c r="D5" s="1">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="1">
+        <v>43</v>
+      </c>
+      <c r="D6" s="1">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="1">
+        <v>12</v>
+      </c>
+      <c r="D7" s="1">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="1">
+        <v>457</v>
+      </c>
+      <c r="D8" s="1">
+        <v>30</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>